<commit_message>
Phase 3: Tasks & Reminders complete
</commit_message>
<xml_diff>
--- a/data/department.xlsx
+++ b/data/department.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="8">
   <si>
     <t>Name</t>
   </si>
@@ -34,6 +34,12 @@
   </si>
   <si>
     <t>Civil Engineering</t>
+  </si>
+  <si>
+    <t>Management Studies</t>
+  </si>
+  <si>
+    <t>Physics</t>
   </si>
 </sst>
 </file>
@@ -365,7 +371,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="36.42578125" customWidth="1"/>
@@ -404,9 +410,25 @@
         <v>2</v>
       </c>
     </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" t="s">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B4">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B6">
       <formula1>"Yes, No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Employee Core field updates, Contact import discoverability, list filters, sort & Excel export
</commit_message>
<xml_diff>
--- a/data/department.xlsx
+++ b/data/department.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="19">
   <si>
     <t>Name</t>
   </si>
@@ -27,9 +27,6 @@
     <t>Yes</t>
   </si>
   <si>
-    <t>Computer Science &amp; Engineering</t>
-  </si>
-  <si>
     <t>Electronics Engineering</t>
   </si>
   <si>
@@ -40,13 +37,49 @@
   </si>
   <si>
     <t>Physics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chemistry </t>
+  </si>
+  <si>
+    <t>Computer Science &amp;  Applications</t>
+  </si>
+  <si>
+    <t>Computer Science &amp;  Engineering</t>
+  </si>
+  <si>
+    <t>Electrical Engineering</t>
+  </si>
+  <si>
+    <t>Electronics Instrumentation &amp; Control</t>
+  </si>
+  <si>
+    <t>Environmental Science</t>
+  </si>
+  <si>
+    <t>Journalism &amp; Mass Communication</t>
+  </si>
+  <si>
+    <t>Library</t>
+  </si>
+  <si>
+    <t>Life Sciences</t>
+  </si>
+  <si>
+    <t>Litrature &amp; Languages</t>
+  </si>
+  <si>
+    <t>Mathematics</t>
+  </si>
+  <si>
+    <t>Mechanical Engineering</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -54,16 +87,35 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <name val="Cambria"/>
+      <family val="1"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Cambria"/>
+      <family val="1"/>
+      <scheme val="major"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -71,12 +123,59 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -371,7 +470,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="36.42578125" customWidth="1"/>
@@ -386,49 +485,137 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
-      <c r="A2" t="s">
+    <row r="2" spans="1:2" ht="15.75">
+      <c r="A2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="15.75">
+      <c r="A3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="15.75">
+      <c r="A4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="15.75">
+      <c r="A5" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="15.75">
+      <c r="A6" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="15.75">
+      <c r="A7" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2">
-      <c r="A4" t="s">
+      <c r="B7" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="31.5">
+      <c r="A8" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="15.75">
+      <c r="A9" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="31.5">
+      <c r="A10" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="15.75">
+      <c r="A11" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="15.75">
+      <c r="A12" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="15.75">
+      <c r="A13" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="15.75">
+      <c r="A14" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B4" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2">
-      <c r="A5" t="s">
+      <c r="B14" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="15.75">
+      <c r="A15" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="15.75">
+      <c r="A16" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="15.75">
+      <c r="A17" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B5" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2">
-      <c r="A6" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6" t="s">
+      <c r="B17" t="s">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B6">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B17">
       <formula1>"Yes, No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>